<commit_message>
Actualizacion pedidos 13.10: Comercial y Fabricacion
</commit_message>
<xml_diff>
--- a/Orden_Fabricacion_MRP_Codiagro.xlsx
+++ b/Orden_Fabricacion_MRP_Codiagro.xlsx
@@ -845,7 +845,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 08/10/2026 07:30</t>
+          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 13/10/2026 07:21</t>
         </is>
       </c>
     </row>
@@ -20782,7 +20782,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 08/10/2026 07:30</t>
+          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 13/10/2026 07:21</t>
         </is>
       </c>
     </row>
@@ -25229,7 +25229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 08/10/2026 07:30</t>
+          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 13/10/2026 07:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix filtro pedidos con fecha nula: incorporados 44 pedidos nuevos del 23.10
</commit_message>
<xml_diff>
--- a/Orden_Fabricacion_MRP_Codiagro.xlsx
+++ b/Orden_Fabricacion_MRP_Codiagro.xlsx
@@ -845,7 +845,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 23/10/2026 08:38</t>
+          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 23/10/2026 08:50</t>
         </is>
       </c>
     </row>
@@ -22390,7 +22390,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 23/10/2026 08:38</t>
+          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 23/10/2026 08:50</t>
         </is>
       </c>
     </row>
@@ -27213,7 +27213,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 23/10/2026 08:38</t>
+          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 23/10/2026 08:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sincronizacion pedidos con fechas asignadas 21.10 y 22.10
</commit_message>
<xml_diff>
--- a/Orden_Fabricacion_MRP_Codiagro.xlsx
+++ b/Orden_Fabricacion_MRP_Codiagro.xlsx
@@ -845,7 +845,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 23/10/2026 08:50</t>
+          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 23/10/2026 08:56</t>
         </is>
       </c>
     </row>
@@ -22390,7 +22390,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 23/10/2026 08:50</t>
+          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 23/10/2026 08:56</t>
         </is>
       </c>
     </row>
@@ -27213,7 +27213,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 23/10/2026 08:50</t>
+          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 23/10/2026 08:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(fullcost): resolver hallazgos auditoria chatgpt 29-10 (seguridad social, ceco 230, controles, capacidad dinamica, validador estricto y 14 pruebas pass)
</commit_message>
<xml_diff>
--- a/Orden_Fabricacion_MRP_Codiagro.xlsx
+++ b/Orden_Fabricacion_MRP_Codiagro.xlsx
@@ -845,7 +845,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 29/10/2026 07:32</t>
+          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 29/10/2026 08:06</t>
         </is>
       </c>
     </row>
@@ -21586,7 +21586,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 29/10/2026 07:32</t>
+          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 29/10/2026 08:06</t>
         </is>
       </c>
     </row>
@@ -26409,7 +26409,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 29/10/2026 07:32</t>
+          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 29/10/2026 08:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(fullcost): resolver segunda auditoria chatgpt 29-10 (subactividad, CECO 410, comparacion JSON/JS, puente materiales, clean rollback)
</commit_message>
<xml_diff>
--- a/Orden_Fabricacion_MRP_Codiagro.xlsx
+++ b/Orden_Fabricacion_MRP_Codiagro.xlsx
@@ -845,7 +845,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 29/10/2026 08:06</t>
+          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 29/10/2026 09:19</t>
         </is>
       </c>
     </row>
@@ -21586,7 +21586,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 29/10/2026 08:06</t>
+          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 29/10/2026 09:19</t>
         </is>
       </c>
     </row>
@@ -26409,7 +26409,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 29/10/2026 08:06</t>
+          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 29/10/2026 09:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(fullcost): resolver auditoria ronda 4 chatgpt (staging estricto, verify_untouched, comparacion exhaustiva comerciales/margenes en js, ss real)
</commit_message>
<xml_diff>
--- a/Orden_Fabricacion_MRP_Codiagro.xlsx
+++ b/Orden_Fabricacion_MRP_Codiagro.xlsx
@@ -845,7 +845,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 29/10/2026 09:19</t>
+          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 29/10/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -21586,7 +21586,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 29/10/2026 09:19</t>
+          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 29/10/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -26409,7 +26409,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 29/10/2026 09:19</t>
+          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 29/10/2026 11:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(fullcost): resolver auditoria ronda 5 chatgpt (sintaxis js en index.html, ruta dinamica base_dir, validacion de sintaxis en validador y prueba en copia)
</commit_message>
<xml_diff>
--- a/Orden_Fabricacion_MRP_Codiagro.xlsx
+++ b/Orden_Fabricacion_MRP_Codiagro.xlsx
@@ -845,7 +845,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 29/10/2026 11:16</t>
+          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 29/10/2026 11:42</t>
         </is>
       </c>
     </row>
@@ -21586,7 +21586,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 29/10/2026 11:16</t>
+          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 29/10/2026 11:42</t>
         </is>
       </c>
     </row>
@@ -26409,7 +26409,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 29/10/2026 11:16</t>
+          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 29/10/2026 11:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(fullcost): resolver 12 puntos de auditoria GPT Astra (transporte REGION, subactividad exacta, cascada dinamica, controles de entrada y sincronizacion BI)
</commit_message>
<xml_diff>
--- a/Orden_Fabricacion_MRP_Codiagro.xlsx
+++ b/Orden_Fabricacion_MRP_Codiagro.xlsx
@@ -845,7 +845,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 29/10/2026 11:42</t>
+          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 29/10/2026 12:42</t>
         </is>
       </c>
     </row>
@@ -21586,7 +21586,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 29/10/2026 11:42</t>
+          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 29/10/2026 12:42</t>
         </is>
       </c>
     </row>
@@ -26409,7 +26409,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 29/10/2026 11:42</t>
+          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 29/10/2026 12:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(fullcost): resolver 12 puntos de auditoria Astra y superar stress suite 100% PASS
- Corregir doble computo de maquila en cascada (-MAQ_CTAS)
- Base industrial NIC 2: tarifas de actividad dependientes de capacidad normal/produccion real (independientes de ventas)
- Desglose de Maquila en UI: reflejar 3.682,80 EUR y 2.751,20 EUR en lugar de ceros
- Puente de conciliacion de margen: cuadre aritmetico exacto (0,00 EUR de desviacion)
- Escalamiento proporcional de coste de planta en detalle analitico (clientes, productos, comerciales)
- Exhaustividad del validador y proteccion en clean_rollback contra activacion incompleta
- Tabla estructurada de conciliacion de perimetros de facturacion en informe final
</commit_message>
<xml_diff>
--- a/Orden_Fabricacion_MRP_Codiagro.xlsx
+++ b/Orden_Fabricacion_MRP_Codiagro.xlsx
@@ -845,7 +845,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 29/10/2026 12:42</t>
+          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 29/10/2026 13:17</t>
         </is>
       </c>
     </row>
@@ -21586,7 +21586,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 29/10/2026 12:42</t>
+          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 29/10/2026 13:17</t>
         </is>
       </c>
     </row>
@@ -26409,7 +26409,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 29/10/2026 12:42</t>
+          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 29/10/2026 13:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(fullcost): resolver invariancia de coste unitario y desacoplar descuentos 706/709
- Eliminar reajuste proporcional de bolsa mensual en ventas: el coste unitario industrial por SKU es estrictamente estandar y constante frente a variaciones de volumen vendido (NIC 2)
- Desacoplar cuentas 706000001 y 709000001 de ventas base para evitar doble computo al actualizar descuentos comerciales en Ajustes_ventas y contabilidad
- Conciliar en el Puente de Margen el coste de actividad activado en variacion de existencias PT (+6.005,79 EUR) con cuadre exacto a 0,00 EUR de desviacion
- Actualizar validador para verificar coherencia entre coste de actividad total y coste absorbido por ventas
</commit_message>
<xml_diff>
--- a/Orden_Fabricacion_MRP_Codiagro.xlsx
+++ b/Orden_Fabricacion_MRP_Codiagro.xlsx
@@ -845,7 +845,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 29/10/2026 13:17</t>
+          <t xml:space="preserve">  Horizonte: Oct 26 (N) + Nov 26 + Dic 26 (3 meses)  |  Ámbito: Global (Nacional + Exportación)  |  Exportación: Siempre Sobre Pedido  |  Fecha Emisión: 29/10/2026 13:40</t>
         </is>
       </c>
     </row>
@@ -21586,7 +21586,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 29/10/2026 13:17</t>
+          <t xml:space="preserve">  Horizonte: Octubre 2026 - Diciembre 2026  |  Total Graneles Químicos a Fabricar en Planta  |  Fecha Emisión: 29/10/2026 13:40</t>
         </is>
       </c>
     </row>
@@ -26409,7 +26409,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 29/10/2026 13:17</t>
+          <t xml:space="preserve">  Premisa de Gestión: Previsiones exclusivamente del Mercado Nacional (España). La exportación se fabricará siempre sobre pedido.  |  Fecha: 29/10/2026 13:40</t>
         </is>
       </c>
     </row>

</xml_diff>